<commit_message>
agentic-qe-mvp: hotel reports and end-to-end guidance use hotel-booking wording
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/flow-1-baseline-CYC-4/09-report/CYC-4-cycle-report.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/flow-1-baseline-CYC-4/09-report/CYC-4-cycle-report.xlsx
@@ -161,7 +161,7 @@
     <t>sri465inno/uc-agentic-quality-engineering@demo/commission-engine (df5203e)</t>
   </si>
   <si>
-    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/commission-engine (df5203e) at 2026-10-02T03:54:15.412Z</t>
+    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/commission-engine (df5203e) at 2026-10-02T04:13:54.623Z</t>
   </si>
   <si>
     <t>ID</t>
@@ -913,7 +913,7 @@
     <t>Priya Shah</t>
   </si>
   <si>
-    <t>2026-10-02T03:54:16.127Z</t>
+    <t>2026-10-02T04:13:55.299Z</t>
   </si>
   <si>
     <t>14 requirements approved; 0 excluded; 1 conflict(s) resolved</t>
@@ -3355,7 +3355,7 @@
         <v>224</v>
       </c>
       <c r="E2" s="2">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F2" s="2"/>
     </row>
@@ -3373,7 +3373,7 @@
         <v>224</v>
       </c>
       <c r="E3" s="2">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F3" s="2"/>
     </row>
@@ -3391,7 +3391,7 @@
         <v>224</v>
       </c>
       <c r="E4" s="2">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F4" s="2"/>
     </row>
@@ -3409,7 +3409,7 @@
         <v>224</v>
       </c>
       <c r="E5" s="2">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F5" s="2"/>
     </row>
@@ -3463,7 +3463,7 @@
         <v>225</v>
       </c>
       <c r="E8" s="2">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F8" s="2"/>
     </row>
@@ -3481,7 +3481,7 @@
         <v>224</v>
       </c>
       <c r="E9" s="2">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F9" s="2"/>
     </row>
@@ -3499,7 +3499,7 @@
         <v>224</v>
       </c>
       <c r="E10" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F10" s="2"/>
     </row>
@@ -3517,7 +3517,7 @@
         <v>224</v>
       </c>
       <c r="E11" s="2">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F11" s="2"/>
     </row>
@@ -3535,7 +3535,7 @@
         <v>224</v>
       </c>
       <c r="E12" s="2">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F12" s="2"/>
     </row>
@@ -3591,7 +3591,7 @@
         <v>224</v>
       </c>
       <c r="E15" s="2">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F15" s="2"/>
     </row>

</xml_diff>